<commit_message>
Update briefs 2026-03-31 08:18 ET
</commit_message>
<xml_diff>
--- a/pitch/stock_pitch_SBAC.xlsx
+++ b/pitch/stock_pitch_SBAC.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -124,11 +124,16 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00F0F4F8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="00F5C542"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -170,6 +175,11 @@
         <fgColor rgb="00E03E3E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003D1010"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -197,7 +207,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -269,7 +279,16 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -720,7 +739,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>$0.00</t>
+          <t>$167.06</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1186,7 +1205,7 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>$2.8B</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -6571,109 +6590,190 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>RISK MATRIX BY CATEGORY</t>
+          <t>THESIS-KILLER RISK</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Risk Description</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Carrier Churn and Lease Non-Renewal: SBA's revenue model depends almost entirely on long-term master lease agreements with a small number of wireless carriers, and any material deterioration in carrier health, merger-driven network consolidation, or aggressive lease renegotiation poses a direct threat to the contracted cash flow that underpins the tower REIT valuation framework. The T-Mobile/Sprin</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="H5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>KEY RISKS &amp; MITIGANTS</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Risk Name</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Probability</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Impact</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Monitoring Metric</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Mitigation</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>WHAT WOULD MAKE US WRONG</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• {'condition': 'US domestic organic tower revenue growth accelerates to above 4.5% annualized for three consecutive quarters, driven by confirmed 5G mid-band densification spending increases disclosed </t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>• {'condition': 'SBAC reduces net debt/EBITDA below 6.0x through a combination of EBITDA growth and asset sale proceeds from remaining international exits, materially reducing refinancing risk and expan</t>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Price Impact %</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Mitigant</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Early Warning</t>
         </is>
       </c>
       <c r="H8" s="2" t="n"/>
     </row>
-    <row r="9">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>• {'condition': 'At least two of the three major US wireless carriers publicly announce multi-year tower amendment programs specifically tied to 5G densification capex, each committing to greater than $</t>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>★ 1</t>
+        </is>
+      </c>
+      <c r="B9" s="27" t="inlineStr">
+        <is>
+          <t>Carrier Churn and Le</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>SBA's revenue model depends almost entirely on long-term master lease agreements</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>-30%</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>SBAC's lease structures are among the most creditor-friendly</t>
+        </is>
+      </c>
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>Quarterly domestic organic revenue growt</t>
         </is>
       </c>
       <c r="H9" s="2" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Leverage Crunch in S</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Tower REITs are structurally high-leverage businesses — SBAC has historically op</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>-25%</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>SBAC's cash flow profile is highly predictable and contracte</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>SBAC reporting net debt/EBITDA above 7.5</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="n"/>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>LEO Satellite Struct</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Low-earth-orbit satellite broadband — led by SpaceX Starlink and soon Amazon Kui</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>-45%</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The credible limiting factor on LEO displacement is physics </t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>SBAC international organic revenue growt</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
@@ -6687,43 +6787,35 @@
       <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>WHAT WOULD MAKE US WRONG</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• {'condition': 'US domestic organic tower revenue growth accelerates to above 4.5% annualized for three consecutive quarters, driven by confirmed 5G mid-band densification spending increases disclosed </t>
+        </is>
+      </c>
       <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>• {'condition': 'SBAC reduces net debt/EBITDA below 6.0x through a combination of EBITDA growth and asset sale proceeds from remaining international exits, materially reducing refinancing risk and expan</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>• {'condition': 'At least two of the three major US wireless carriers publicly announce multi-year tower amendment programs specifically tied to 5G densification capex, each committing to greater than $</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
@@ -7367,12 +7459,14 @@
       <c r="H80" s="2" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A8:G8"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A4:G5"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A7:G7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>